<commit_message>
Fix label clipping in invoice/receipt info table (PDF mode)
PDF mode scales every font 15% but never adjusted rows 8/10 (fixed
height=16, sized for the original 14pt font) or column I's width,
so "Terms"/"Due Date" clipped at the top and "Invoice No."/
"เงื่อนไขชำระ(วัน)" clipped on the right once enlarged.

- Templates: cleared the fixed height on rows 8 & 10 so they auto-fit
  like their neighbors (5,6,7,9) already did.
- fill_invoice.py: extended the existing shrink-to-fit fix (already
  applied to I9/I10 for this same symptom) to I5 and I7 too.

Verified through the real pipeline (fill_invoice -> xlsx_to_pdf.ps1 ->
render) for invoice and both receipt pages: labels fully readable,
still fits on one page, zero formula errors.
</commit_message>
<xml_diff>
--- a/server/templates/invoice-template.xlsx
+++ b/server/templates/invoice-template.xlsx
@@ -1935,7 +1935,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1">
+    <row r="8">
       <c r="A8" s="56" t="n"/>
       <c r="B8" s="68" t="n"/>
       <c r="C8" s="68" t="n"/>
@@ -1986,7 +1986,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10">
       <c r="A10" s="56" t="n"/>
       <c r="D10" s="47" t="n"/>
       <c r="E10" s="47" t="n"/>

</xml_diff>